<commit_message>
feat: update new projects for PJM area
</commit_message>
<xml_diff>
--- a/reference/us_reconductoring_projects.xlsx
+++ b/reference/us_reconductoring_projects.xlsx
@@ -25,13 +25,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +48,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -52,15 +65,27 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -2835,11 +2860,11 @@
     <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
     <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="110" customWidth="1" min="11" max="11"/>
+    <col width="24.005" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
+    <col width="14.005" bestFit="1" customWidth="1" style="2" min="8" max="8"/>
+    <col width="14.005" bestFit="1" customWidth="1" style="2" min="9" max="9"/>
+    <col width="14.005" bestFit="1" customWidth="1" style="2" min="10" max="10"/>
+    <col width="110.005" bestFit="1" customWidth="1" style="6" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
@@ -2893,59 +2918,60 @@
           <t>Planned Year</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17.25" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="17.25" customFormat="1" customHeight="1" s="4">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Cayuga - Wolf Creek 345 kV baseline transmission upgrade</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>CAYUGA</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>WOLF CREEK</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Baseline reliability upgrade</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>345</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>MISO</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Duke Energy Indiana</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Coordinated MISO baseline transmission upgrades rebuild and reconductor the 345 kV lines connecting Cayuga, Nucor, and Wolf Creek. The program includes a $96 million Cayuga-to-Nucor rebuild and a $49 million Nucor-to-Wolf Creek rebuild targeted for completion by June 2029.</t>
         </is>
@@ -2982,6 +3008,11 @@
           <t>MISO</t>
         </is>
       </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="6" t="n"/>
     </row>
     <row r="4" ht="17.25" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -3014,6 +3045,11 @@
           <t>MISO</t>
         </is>
       </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="6" t="n"/>
     </row>
     <row r="5" ht="17.25" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -3046,6 +3082,11 @@
           <t>MISO</t>
         </is>
       </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="6" t="n"/>
     </row>
     <row r="6" ht="17.25" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -3078,6 +3119,11 @@
           <t>MISO</t>
         </is>
       </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="6" t="n"/>
     </row>
     <row r="7" ht="17.25" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -3110,6 +3156,11 @@
           <t>MISO</t>
         </is>
       </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="6" t="n"/>
     </row>
     <row r="8" ht="17.25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -3142,6 +3193,11 @@
           <t>MISO</t>
         </is>
       </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3336,20 +3392,21 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
+    <col width="72" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
     <col width="20.57642857142857" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
     <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
-    <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
+    <col width="52" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
     <col width="12.43357142857143" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="110" customWidth="1" min="11" max="11"/>
+    <col width="24" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
+    <col width="16" bestFit="1" customWidth="1" style="2" min="8" max="8"/>
+    <col width="14" bestFit="1" customWidth="1" style="2" min="9" max="9"/>
+    <col width="14.005" bestFit="1" customWidth="1" style="2" min="10" max="10"/>
+    <col width="110" bestFit="1" customWidth="1" style="6" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
@@ -3403,9 +3460,14 @@
           <t>Planned Year</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Description</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Rating</t>
         </is>
       </c>
     </row>
@@ -3440,6 +3502,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="6" t="n"/>
     </row>
     <row r="3" ht="17.25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -3472,6 +3539,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="6" t="n"/>
     </row>
     <row r="4" ht="17.25" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -3504,6 +3576,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="6" t="n"/>
     </row>
     <row r="5" ht="17.25" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -3536,6 +3613,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="6" t="n"/>
     </row>
     <row r="6" ht="17.25" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -3568,6 +3650,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="6" t="n"/>
     </row>
     <row r="7" ht="17.25" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -3600,6 +3687,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="6" t="n"/>
     </row>
     <row r="8" ht="17.25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -3632,6 +3724,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="6" t="n"/>
     </row>
     <row r="9" ht="17.25" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -3664,8 +3761,13 @@
           <t>PJM</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="17.25" customHeight="1">
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="28.5" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>LICK - JEFFERSON 69 kV reconductoring project</t>
@@ -3696,7 +3798,11 @@
           <t>PJM</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>Reconductoring project for the existing LICK - JEFFERSON 69 kV transmission line in the PJM region. Utility, distance, rating, cost, status, and planned-year details are not available in the current project source data.</t>
         </is>
@@ -3733,54 +3839,60 @@
           <t>PJM</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="17.25" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="84.75" customFormat="1" customHeight="1" s="4">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Chesterfield - Tyler 230 kV transmission rebuild and reconductor project</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>CHESTERFIELD</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>TYLER</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Supplemental transmission planning reliability upgrade</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>230</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>PJM</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Dominion Energy</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>2.9</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Rebuild and reconductor 2.9 miles of overhead transmission line from the Chesterfield Substation to just south of the Tyler Substation in Chesterfield County, Virginia. The operating voltage will remain 230 kV while new structures and higher-capacity conductors replace aging infrastructure, increase ampacity, and support regional data center growth, local generation, and reliability needs through Dominion Energy's supplemental transmission planning process.</t>
         </is>
@@ -3817,6 +3929,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="6" t="n"/>
     </row>
     <row r="14" ht="17.25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -3849,6 +3966,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="6" t="n"/>
     </row>
     <row r="15" ht="17.25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -3881,6 +4003,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="6" t="n"/>
     </row>
     <row r="16" ht="17.25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -3913,6 +4040,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="6" t="n"/>
     </row>
     <row r="17" ht="17.25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -3945,6 +4077,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="6" t="n"/>
     </row>
     <row r="18" ht="17.25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -3977,6 +4114,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="6" t="n"/>
     </row>
     <row r="19" ht="17.25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -4009,6 +4151,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="6" t="n"/>
     </row>
     <row r="20" ht="17.25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -4041,6 +4188,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="6" t="n"/>
     </row>
     <row r="21" ht="17.25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -4073,6 +4225,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="6" t="n"/>
     </row>
     <row r="22" ht="17.25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -4105,6 +4262,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="6" t="n"/>
     </row>
     <row r="23" ht="17.25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -4137,6 +4299,11 @@
           <t>PJM</t>
         </is>
       </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="6" t="n"/>
     </row>
     <row r="24" ht="17.25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -4167,6 +4334,494 @@
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>PJM</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Leroy Center - Mayfield Q1 138 kV reconductoring need</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>LEROY CENTER</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>MAYFIELD</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Existing reconductoring</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>ATSI</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>The Leroy Center - Mayfield Q1 138 kV line is approximately 16.1 miles long and was originally constructed in the mid-1940s. The Leroy Center - Pawnee Tap Q1 138 kV section, approximately 8.4 miles, is being reconductored under RTEP project B3152. The remaining Pawnee Tap - Mayfield Q1 138 kV section is approximately 7.7 miles, with aging structures, conductors, and hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Powell County - Zachariah 69 kV reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>POWELL COUNTY</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>ZACHARIAH</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>EKPC</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>16.85</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>The 16.85-mile Powell County - Zachariah 69 kV line was built in 1954. EKPC identified the line for structural loading concerns associated with single wood-pole structures and 556.5 ACSR wire or larger. The source notes that many lines in the program have previously been reconductored with larger wire without corresponding structural design work; alternatives will be developed to address the remaining structural concerns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Rob Park - Lincoln 138 kV line rebuild and reconductoring</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>ROB PARK</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>LINCOLN</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Existing line rebuild and reconductoring</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>10.9 / 7.8</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>The Robison Park - Lincoln 138 kV line is approximately 10.9/7.8 miles long and has 44 structures with open conditions, including rusted legs, damaged insulators, and rusted shield wire. The line does not meet current AEP structural-strength or shield-angle requirements. The upper tower sections were replaced and reconductored in 1968 for 138 kV operation, while the lower sections and foundations date to the original 1928 installation. The remaining 3.1 miles are covered under AEP-2019-IM038 and will be addressed through a future solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Remington CT - Elk Run 230 kV Line 2114 reconductoring</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>REMINGTON CT</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>ELK RUN</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Approved baseline reconductoring</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Dominion Energy</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>3.46</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>Under approved baseline solution b3689.1, reconductor approximately 3.46 miles of 230 kV Line 2114 from Remington CT to Elk Run using higher-capacity conductor to achieve an expected 1573 MVA rating.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>1573 MVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Elk Run - Rollins Ford 230 kV Line 2114 reconductoring</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>ELK RUN</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>ROLLINS FORD</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Approved baseline reconductoring</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Dominion Energy</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>19.71</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>Under approved baseline solution b3689.1, reconductor approximately 19.71 miles of 230 kV Line 2114 from Elk Run to Rollins Ford using higher-capacity conductor to achieve an expected 1573 MVA rating.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>1573 MVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Rollins Ford - Gainesville 230 kV Line 2222 reconductoring</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>ROLLINS FORD</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>GAINESVILLE</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Approved baseline reconductoring</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Dominion Energy</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>Under approved baseline solution b3689.1, reconductor approximately 1.11 miles of 230 kV Line 2222 from Rollins Ford to Gainesville using higher-capacity conductor to achieve an expected 1573 MVA rating.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>1573 MVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Elizabethtown - Central Hardin - Stephensburg 69 kV reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ELIZABETHTOWN</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>STEPHENSBURG</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>EKPC</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>EKPC identified the 11.7-mile Elizabethtown - Central Hardin - Stephensburg 69 kV line sections for structural loading concerns. The source notes that many lines in the program have been reconductored with larger wire while receiving limited structural design work; alternatives will be developed to address the structural concerns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Elizabethtown - Patriot Parkway - Vine Grove 69 kV reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>ELIZABETHTOWN</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>VINE GROVE</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>EKPC</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>7.45</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>EKPC identified the 7.45-mile Elizabethtown - Patriot Parkway - Vine Grove 69 kV line sections for structural loading concerns. The source notes that many lines in the program have been reconductored with larger wire while receiving limited structural design work; alternatives will be developed to address the structural concerns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Windsor - Somerset 69 kV reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>WINDSOR</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>SOMERSET</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Reconductoring-related structural reliability upgrade</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>PJM</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>EKPC</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>18.97</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>EKPC identified the 18.97-mile Windsor - Somerset 69 kV line sections for structural loading concerns. The source notes that many lines in the program have been reconductored with larger wire while receiving limited structural design work; alternatives will be developed to address the structural concerns.</t>
         </is>
       </c>
     </row>

</xml_diff>